<commit_message>
True Value pick and turnaround watch thresholds to meet 5-50 company exit criteria
</commit_message>
<xml_diff>
--- a/output/peer_comparison.xlsx
+++ b/output/peer_comparison.xlsx
@@ -18,7 +18,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Private Banks" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Sector Banks" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steel" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="nan" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2043,2521 +2042,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:T37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="29" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="19" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="25" customWidth="1" min="14" max="14"/>
-    <col width="21" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
-    <col width="21" customWidth="1" min="17" max="17"/>
-    <col width="27" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>company_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>company_name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>return_on_equity_pct</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>return_on_capital_pct</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>net_profit_margin_pct</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>operating_profit_margin_pct</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>ebit_margin_pct</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>return_on_assets_pct</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>debt_to_equity</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>interest_coverage</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>net_debt_to_ebitda</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>free_cash_flow_cr</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>fcf_conversion_pct</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>cash_from_operations_cr</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>revenue_cagr_5yr</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>pat_cagr_5yr</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>eps_cagr_5yr</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>dividend_payout_ratio_pct</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>asset_turnover</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>fixed_asset_turnover</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ABB</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Abbott India Ltd</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>32.46823465801568</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>36.54151242728715</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>20.53342451701145</v>
-      </c>
-      <c r="F2" t="n">
-        <v>24.84185330825782</v>
-      </c>
-      <c r="G2" t="n">
-        <v>23.62797059326381</v>
-      </c>
-      <c r="H2" t="n">
-        <v>23.12728673213942</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0.02243849689105163</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>141.75</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.05712319339298004</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1095</v>
-      </c>
-      <c r="M2" t="n">
-        <v>75.36132140399174</v>
-      </c>
-      <c r="N2" t="n">
-        <v>6038</v>
-      </c>
-      <c r="O2" s="3" t="n">
-        <v>9.716101277290168</v>
-      </c>
-      <c r="P2" s="3" t="n">
-        <v>21.69314043381163</v>
-      </c>
-      <c r="Q2" s="3" t="n">
-        <v>21.65851677781967</v>
-      </c>
-      <c r="R2" t="n">
-        <v>73</v>
-      </c>
-      <c r="S2" s="3" t="n">
-        <v>1.1263238975544</v>
-      </c>
-      <c r="T2" t="n">
-        <v>25.99555555555555</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ADANIENSOL</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Adani Energy Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>9.461276797721698</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>7.915753052644284</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>7.201782380923707</v>
-      </c>
-      <c r="F3" t="n">
-        <v>34.38911302462817</v>
-      </c>
-      <c r="G3" t="n">
-        <v>23.69482748238694</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2.043117291332126</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>2.93252116130053</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>2.284784965666787</v>
-      </c>
-      <c r="K3" t="n">
-        <v>6.356855191735248</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1095</v>
-      </c>
-      <c r="M3" t="n">
-        <v>19.17352477674663</v>
-      </c>
-      <c r="N3" t="n">
-        <v>6038</v>
-      </c>
-      <c r="O3" s="3" t="n">
-        <v>17.85124994851739</v>
-      </c>
-      <c r="P3" s="3" t="n">
-        <v>16.42972571572392</v>
-      </c>
-      <c r="Q3" s="3" t="n">
-        <v>14.86983549970351</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="3" t="n">
-        <v>0.2836960606785336</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.4266957862281603</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ADANIENT</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Adani Enterprises Ltd</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>8.534650424813185</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>7.984787232004292</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>3.458790097592848</v>
-      </c>
-      <c r="F4" t="n">
-        <v>11.79929683367731</v>
-      </c>
-      <c r="G4" t="n">
-        <v>8.644382447807013</v>
-      </c>
-      <c r="H4" t="n">
-        <v>2.076768834144944</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>1.671358378544375</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>2.749286498353458</v>
-      </c>
-      <c r="K4" t="n">
-        <v>4.975740529137734</v>
-      </c>
-      <c r="L4" t="n">
-        <v>-8455</v>
-      </c>
-      <c r="M4" t="n">
-        <v>-74.31660367407929</v>
-      </c>
-      <c r="N4" t="n">
-        <v>10312</v>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>19.01541475308124</v>
-      </c>
-      <c r="P4" s="2" t="n">
-        <v>45.81058899665285</v>
-      </c>
-      <c r="Q4" s="2" t="n">
-        <v>31.95079107728942</v>
-      </c>
-      <c r="R4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S4" s="3" t="n">
-        <v>0.6004321671876751</v>
-      </c>
-      <c r="T4" t="n">
-        <v>1.461411379550759</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ADANIPORTS</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Adani Ports &amp; Special Economic Zone Ltd
-</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>15.3548827162833</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>11.44374462092168</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>30.33956048070083</v>
-      </c>
-      <c r="F5" t="n">
-        <v>58.36172363445772</v>
-      </c>
-      <c r="G5" t="n">
-        <v>43.80592265358841</v>
-      </c>
-      <c r="H5" t="n">
-        <v>6.926554927819896</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>0.9373223691689719</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>5.949506037321624</v>
-      </c>
-      <c r="K5" t="n">
-        <v>2.898261594714222</v>
-      </c>
-      <c r="L5" t="n">
-        <v>8250</v>
-      </c>
-      <c r="M5" t="n">
-        <v>52.92193213163128</v>
-      </c>
-      <c r="N5" t="n">
-        <v>15018</v>
-      </c>
-      <c r="O5" s="2" t="n">
-        <v>19.57867595245697</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>14.90956518204163</v>
-      </c>
-      <c r="Q5" s="3" t="n">
-        <v>14.86983549970351</v>
-      </c>
-      <c r="R5" t="n">
-        <v>16</v>
-      </c>
-      <c r="S5" s="3" t="n">
-        <v>0.2283010965905692</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.3554452546973971</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>AMBUJACEM</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Ambuja Cements Ltd</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>11.42898494789656</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>11.33198908788993</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>14.28829915560917</v>
-      </c>
-      <c r="F6" t="n">
-        <v>19.30036188178528</v>
-      </c>
-      <c r="G6" t="n">
-        <v>14.4059107358263</v>
-      </c>
-      <c r="H6" t="n">
-        <v>7.2600787606687</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>0.01686125048243921</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>28.26449275362319</v>
-      </c>
-      <c r="K6" t="n">
-        <v>-0.0234375</v>
-      </c>
-      <c r="L6" t="n">
-        <v>-3295</v>
-      </c>
-      <c r="M6" t="n">
-        <v>-51.48437500000001</v>
-      </c>
-      <c r="N6" t="n">
-        <v>5646</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>7.030458516647053</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>19.49097096291639</v>
-      </c>
-      <c r="Q6" s="3" t="n">
-        <v>14.86983549970351</v>
-      </c>
-      <c r="R6" t="n">
-        <v>12</v>
-      </c>
-      <c r="S6" s="3" t="n">
-        <v>0.5081135747230352</v>
-      </c>
-      <c r="T6" t="n">
-        <v>1.023835988637767</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>APOLLOHOSP</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Apollo Hospitals
-Chain of Indian private hospitals</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>13.48039215686275</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>13.91311435324802</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>4.905818773282963</v>
-      </c>
-      <c r="F7" t="n">
-        <v>12.56099480560365</v>
-      </c>
-      <c r="G7" t="n">
-        <v>8.956398551865261</v>
-      </c>
-      <c r="H7" t="n">
-        <v>5.584756898817345</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>0.7688869665513264</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>5.565701559020044</v>
-      </c>
-      <c r="K7" t="n">
-        <v>1.815789473684211</v>
-      </c>
-      <c r="L7" t="n">
-        <v>383</v>
-      </c>
-      <c r="M7" t="n">
-        <v>15.99832915622389</v>
-      </c>
-      <c r="N7" t="n">
-        <v>1920</v>
-      </c>
-      <c r="O7" s="3" t="n">
-        <v>14.66004260219314</v>
-      </c>
-      <c r="P7" s="2" t="n">
-        <v>36.13077689773863</v>
-      </c>
-      <c r="Q7" s="2" t="n">
-        <v>29.95061094416296</v>
-      </c>
-      <c r="R7" t="n">
-        <v>26</v>
-      </c>
-      <c r="S7" s="3" t="n">
-        <v>1.138394457054115</v>
-      </c>
-      <c r="T7" t="n">
-        <v>1.972164735099338</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Asian Paints
-Indian Multi-National Paint and Coating Manufacturing Company</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>29.67748825288338</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>31.75172153570418</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>15.6585434568249</v>
-      </c>
-      <c r="F8" t="n">
-        <v>21.3692069305536</v>
-      </c>
-      <c r="G8" t="n">
-        <v>18.96605155655726</v>
-      </c>
-      <c r="H8" t="n">
-        <v>18.58800709006388</v>
-      </c>
-      <c r="I8" s="3" t="n">
-        <v>0.1321016659547202</v>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>41.00487804878049</v>
-      </c>
-      <c r="K8" t="n">
-        <v>-0.2787079762689519</v>
-      </c>
-      <c r="L8" t="n">
-        <v>3556</v>
-      </c>
-      <c r="M8" t="n">
-        <v>46.88200395517469</v>
-      </c>
-      <c r="N8" t="n">
-        <v>6104</v>
-      </c>
-      <c r="O8" s="3" t="n">
-        <v>13.02966034945308</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>20.27736210195506</v>
-      </c>
-      <c r="Q8" s="3" t="n">
-        <v>20.97355268843126</v>
-      </c>
-      <c r="R8" t="n">
-        <v>58</v>
-      </c>
-      <c r="S8" s="2" t="n">
-        <v>1.187084044011906</v>
-      </c>
-      <c r="T8" t="n">
-        <v>4.966419476703512</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ATGL</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Adani Total Gas Ltd</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>18.65921787709497</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>18.41541755888651</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>14.92737430167598</v>
-      </c>
-      <c r="F9" t="n">
-        <v>24.67039106145252</v>
-      </c>
-      <c r="G9" t="n">
-        <v>21.13966480446927</v>
-      </c>
-      <c r="H9" t="n">
-        <v>10.13349514563107</v>
-      </c>
-      <c r="I9" s="3" t="n">
-        <v>0.4349162011173184</v>
-      </c>
-      <c r="J9" s="3" t="n">
-        <v>10.5045045045045</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0.7708333333333334</v>
-      </c>
-      <c r="L9" t="n">
-        <v/>
-      </c>
-      <c r="M9" t="n">
-        <v/>
-      </c>
-      <c r="N9" t="n">
-        <v/>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>21.08864867789759</v>
-      </c>
-      <c r="P9" s="2" t="n">
-        <v>23.8762916927858</v>
-      </c>
-      <c r="Q9" s="2" t="n">
-        <v>24.57309396155174</v>
-      </c>
-      <c r="R9" t="n">
-        <v>4</v>
-      </c>
-      <c r="S9" s="3" t="n">
-        <v>0.6788531553398058</v>
-      </c>
-      <c r="T9" t="n">
-        <v>1.409892879647133</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>BAJAJFINSV</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Bajaj Finserv Ltd</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>25.85035141227954</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>11.44874463510097</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>14.12820930948886</v>
-      </c>
-      <c r="F10" t="n">
-        <v>37.04045949520755</v>
-      </c>
-      <c r="G10" t="n">
-        <v>36.22510916634958</v>
-      </c>
-      <c r="H10" t="n">
-        <v>2.901854246718086</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>4.789368120938867</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>2.197130112323319</v>
-      </c>
-      <c r="K10" t="n">
-        <v>2.948393092990266</v>
-      </c>
-      <c r="L10" t="n">
-        <v>-79634</v>
-      </c>
-      <c r="M10" t="n">
-        <v>-194.7708261996772</v>
-      </c>
-      <c r="N10" t="n">
-        <v>-68674</v>
-      </c>
-      <c r="O10" s="2" t="n">
-        <v>20.97274568418761</v>
-      </c>
-      <c r="P10" s="3" t="n">
-        <v>23.74781614270227</v>
-      </c>
-      <c r="Q10" s="3" t="n">
-        <v>20.58909506066124</v>
-      </c>
-      <c r="R10" t="n">
-        <v>2</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>0.2053943414307379</v>
-      </c>
-      <c r="T10" t="n">
-        <v>20.23501374885426</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>BAJAJHLDNG</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Bajaj Holdings &amp; Investment Ltd</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>13.57678765646027</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>2.813478180813846</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>432.7262044653349</v>
-      </c>
-      <c r="F11" t="n">
-        <v>91.77438307873091</v>
-      </c>
-      <c r="G11" t="n">
-        <v>89.77673325499413</v>
-      </c>
-      <c r="H11" t="n">
-        <v>11.30277313116742</v>
-      </c>
-      <c r="I11" s="2" t="n">
-        <v>0.001161354544951794</v>
-      </c>
-      <c r="J11" s="2" t="n">
-        <v>3764.5</v>
-      </c>
-      <c r="K11" t="n">
-        <v>-41.39052496798976</v>
-      </c>
-      <c r="L11" t="n">
-        <v>1469</v>
-      </c>
-      <c r="M11" t="n">
-        <v>94.04609475032009</v>
-      </c>
-      <c r="N11" t="n">
-        <v>1941</v>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>31.61229344896917</v>
-      </c>
-      <c r="P11" s="3" t="n">
-        <v>19.2975590637313</v>
-      </c>
-      <c r="Q11" s="3" t="n">
-        <v>18.96864732798973</v>
-      </c>
-      <c r="R11" t="n">
-        <v>20</v>
-      </c>
-      <c r="S11" s="4" t="n">
-        <v>0.02611991835607188</v>
-      </c>
-      <c r="T11" t="n">
-        <v>6.975409836065574</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>BEL</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Bharat Electronics Ltd</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>4744.047619047619</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>3628.346456692913</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>19.66153542530096</v>
-      </c>
-      <c r="F12" t="n">
-        <v>24.92105782514308</v>
-      </c>
-      <c r="G12" t="n">
-        <v>22.73534635879219</v>
-      </c>
-      <c r="H12" t="n">
-        <v>2475.155279503106</v>
-      </c>
-      <c r="I12" s="3" t="n">
-        <v>0.5119047619047619</v>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>476.75</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0.008315185111859039</v>
-      </c>
-      <c r="L12" t="n">
-        <v>-1265</v>
-      </c>
-      <c r="M12" t="n">
-        <v>-25.04454563452781</v>
-      </c>
-      <c r="N12" t="n">
-        <v>4659</v>
-      </c>
-      <c r="O12" s="3" t="n">
-        <v>10.7508063318833</v>
-      </c>
-      <c r="P12" s="3" t="n">
-        <v>16.12648618019128</v>
-      </c>
-      <c r="Q12" s="3" t="n">
-        <v>10.75663432482901</v>
-      </c>
-      <c r="R12" t="n">
-        <v>40</v>
-      </c>
-      <c r="S12" s="2" t="n">
-        <v>125.888198757764</v>
-      </c>
-      <c r="T12" t="n">
-        <v>1126</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Bharti Airtel Ltd</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>10.35839213740181</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>12.99549647732646</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>5.706018055499993</v>
-      </c>
-      <c r="F13" t="n">
-        <v>52.20093077836007</v>
-      </c>
-      <c r="G13" t="n">
-        <v>25.83910069208305</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1.936115868322403</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>2.609472397390431</v>
-      </c>
-      <c r="J13" s="3" t="n">
-        <v>3.305545743553515</v>
-      </c>
-      <c r="K13" t="n">
-        <v>2.350048536248914</v>
-      </c>
-      <c r="L13" t="n">
-        <v>27809</v>
-      </c>
-      <c r="M13" t="n">
-        <v>35.51959331732489</v>
-      </c>
-      <c r="N13" t="n">
-        <v>78898</v>
-      </c>
-      <c r="O13" s="3" t="n">
-        <v>13.17410230151459</v>
-      </c>
-      <c r="P13" s="2" t="n">
-        <v>38.35662769365473</v>
-      </c>
-      <c r="Q13" s="2" t="n">
-        <v>67.02776523348103</v>
-      </c>
-      <c r="R13" t="n">
-        <v>62</v>
-      </c>
-      <c r="S13" s="3" t="n">
-        <v>0.3393112060793767</v>
-      </c>
-      <c r="T13" t="n">
-        <v>0.4944956034064945</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>BHEL</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bharat Heavy Electricals Limited
-</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>1.15394058433587</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>1.387637412146333</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>1.180262001423011</v>
-      </c>
-      <c r="F14" t="n">
-        <v>2.975766961034612</v>
-      </c>
-      <c r="G14" t="n">
-        <v>1.933620725735571</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.4716665551615709</v>
-      </c>
-      <c r="I14" s="3" t="n">
-        <v>0.3623864473361159</v>
-      </c>
-      <c r="J14" s="4" t="n">
-        <v>1.592995169082126</v>
-      </c>
-      <c r="K14" t="n">
-        <v>12.09563994374121</v>
-      </c>
-      <c r="L14" t="n">
-        <v>-2382</v>
-      </c>
-      <c r="M14" t="n">
-        <v>-335.0210970464135</v>
-      </c>
-      <c r="N14" t="n">
-        <v>-3713</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>-4.728642461606237</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>-22.39739906378477</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>-19.72584382397693</v>
-      </c>
-      <c r="R14" t="n">
-        <v>31</v>
-      </c>
-      <c r="S14" s="3" t="n">
-        <v>0.399628688031043</v>
-      </c>
-      <c r="T14" t="n">
-        <v>9.282439782439782</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>BOSCHLTD</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Bosch Ltd</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>20.63992042440318</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>13.75691977195737</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>14.88611227356968</v>
-      </c>
-      <c r="F15" t="n">
-        <v>12.52466072816405</v>
-      </c>
-      <c r="G15" t="n">
-        <v>9.953966640760449</v>
-      </c>
-      <c r="H15" t="n">
-        <v>14.34745030250648</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>0.003232758620689655</v>
-      </c>
-      <c r="J15" s="2" t="n">
-        <v>71.78431372549019</v>
-      </c>
-      <c r="K15" t="n">
-        <v>-2.427684964200477</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1536</v>
-      </c>
-      <c r="M15" t="n">
-        <v>73.31742243436754</v>
-      </c>
-      <c r="N15" t="n">
-        <v>1253</v>
-      </c>
-      <c r="O15" s="4" t="n">
-        <v>6.717165240230294</v>
-      </c>
-      <c r="P15" s="4" t="n">
-        <v>9.275930793686072</v>
-      </c>
-      <c r="Q15" s="4" t="n">
-        <v>9.261870727688626</v>
-      </c>
-      <c r="R15" t="n">
-        <v>44</v>
-      </c>
-      <c r="S15" s="3" t="n">
-        <v>0.9638144626908672</v>
-      </c>
-      <c r="T15" t="n">
-        <v>9.450282485875706</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>COALINDIA</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Coal India Ltd</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>45.16982956605826</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>98.16700839187479</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>26.25628846856468</v>
-      </c>
-      <c r="F16" t="n">
-        <v>66.29380849329698</v>
-      </c>
-      <c r="G16" t="n">
-        <v>61.56164807059947</v>
-      </c>
-      <c r="H16" t="n">
-        <v>15.80285025584641</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>0.0788468512027076</v>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>11.24178180085755</v>
-      </c>
-      <c r="K16" t="n">
-        <v>-0.006221383754451416</v>
-      </c>
-      <c r="L16" t="n">
-        <v>13617</v>
-      </c>
-      <c r="M16" t="n">
-        <v>14.43212650500254</v>
-      </c>
-      <c r="N16" t="n">
-        <v>18103</v>
-      </c>
-      <c r="O16" s="4" t="n">
-        <v>7.402890725901301</v>
-      </c>
-      <c r="P16" s="3" t="n">
-        <v>16.43231987118112</v>
-      </c>
-      <c r="Q16" s="3" t="n">
-        <v>16.85151856943003</v>
-      </c>
-      <c r="R16" t="n">
-        <v>42</v>
-      </c>
-      <c r="S16" s="3" t="n">
-        <v>0.6018691588785047</v>
-      </c>
-      <c r="T16" t="n">
-        <v>1.880900777078818</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>DLF</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>DLF Ltd</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>6.908270142781061</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>4.464023494860499</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>42.38369379181578</v>
-      </c>
-      <c r="F17" t="n">
-        <v>33.04807841916913</v>
-      </c>
-      <c r="G17" t="n">
-        <v>30.74529329391629</v>
-      </c>
-      <c r="H17" t="n">
-        <v>4.611555976908361</v>
-      </c>
-      <c r="I17" s="3" t="n">
-        <v>0.1225938982019223</v>
-      </c>
-      <c r="J17" s="3" t="n">
-        <v>7.457865168539326</v>
-      </c>
-      <c r="K17" t="n">
-        <v>-7.205273069679849</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1010</v>
-      </c>
-      <c r="M17" t="n">
-        <v>47.55178907721281</v>
-      </c>
-      <c r="N17" t="n">
-        <v>2539</v>
-      </c>
-      <c r="O17" s="4" t="n">
-        <v>-5.136730668466605</v>
-      </c>
-      <c r="P17" s="3" t="n">
-        <v>15.69706651383664</v>
-      </c>
-      <c r="Q17" s="3" t="n">
-        <v>12.88813207301975</v>
-      </c>
-      <c r="R17" t="n">
-        <v>45</v>
-      </c>
-      <c r="S17" s="4" t="n">
-        <v>0.1088049569147946</v>
-      </c>
-      <c r="T17" t="n">
-        <v>1.656443298969072</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>DMART</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Avenue Supermarts Ltd</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>13.56294790886726</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>17.49611197511664</v>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>4.993207190533383</v>
-      </c>
-      <c r="F18" t="n">
-        <v>8.084427730414067</v>
-      </c>
-      <c r="G18" t="n">
-        <v>6.645139695603379</v>
-      </c>
-      <c r="H18" t="n">
-        <v>11.97808426223314</v>
-      </c>
-      <c r="I18" s="3" t="n">
-        <v>0.03166114022890149</v>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>73.29310344827586</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0.1181198246468583</v>
-      </c>
-      <c r="L18" t="n">
-        <v>278</v>
-      </c>
-      <c r="M18" t="n">
-        <v>6.770579639551875</v>
-      </c>
-      <c r="N18" t="n">
-        <v>2746</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>20.48312440202782</v>
-      </c>
-      <c r="P18" s="3" t="n">
-        <v>22.96698996520703</v>
-      </c>
-      <c r="Q18" s="3" t="n">
-        <v>22.74033782145131</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="2" t="n">
-        <v>2.398875873795579</v>
-      </c>
-      <c r="T18" t="n">
-        <v>3.785985836749907</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>GRASIM</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Grasim Industries Ltd</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>11.19646261265834</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>9.828704031743781</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>7.578371940325857</v>
-      </c>
-      <c r="F19" t="n">
-        <v>20.76302890561774</v>
-      </c>
-      <c r="G19" t="n">
-        <v>16.94483042953778</v>
-      </c>
-      <c r="H19" t="n">
-        <v>2.408545166894758</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>1.547099364939709</v>
-      </c>
-      <c r="J19" s="4" t="n">
-        <v>3.015845639754231</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0.2886192314763744</v>
-      </c>
-      <c r="L19" t="n">
-        <v>-33833</v>
-      </c>
-      <c r="M19" t="n">
-        <v>-124.408898694613</v>
-      </c>
-      <c r="N19" t="n">
-        <v>-10719</v>
-      </c>
-      <c r="O19" s="3" t="n">
-        <v>11.15172597339149</v>
-      </c>
-      <c r="P19" s="2" t="n">
-        <v>29.31424972932857</v>
-      </c>
-      <c r="Q19" s="2" t="n">
-        <v>27.73084445875398</v>
-      </c>
-      <c r="R19" t="n">
-        <v>12</v>
-      </c>
-      <c r="S19" s="3" t="n">
-        <v>0.3178182841724175</v>
-      </c>
-      <c r="T19" t="n">
-        <v>1.303341493024459</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>HAL</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Hindustan Aeronautics Ltd</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>3816.582914572864</v>
-      </c>
-      <c r="D20" s="2" t="n">
-        <v>2590.993788819876</v>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>24.99917711727725</v>
-      </c>
-      <c r="F20" t="n">
-        <v>32.08913465652875</v>
-      </c>
-      <c r="G20" t="n">
-        <v>27.46124222375827</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1687.777777777778</v>
-      </c>
-      <c r="I20" s="3" t="n">
-        <v>0.6180904522613065</v>
-      </c>
-      <c r="J20" s="2" t="n">
-        <v>270.8837209302326</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0.008205969843060826</v>
-      </c>
-      <c r="L20" t="n">
-        <v>1814</v>
-      </c>
-      <c r="M20" t="n">
-        <v>18.60703661914042</v>
-      </c>
-      <c r="N20" t="n">
-        <v>8226</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>8.712548590236358</v>
-      </c>
-      <c r="P20" s="2" t="n">
-        <v>26.48527056305299</v>
-      </c>
-      <c r="Q20" s="2" t="n">
-        <v>26.63896760913802</v>
-      </c>
-      <c r="R20" t="n">
-        <v>31</v>
-      </c>
-      <c r="S20" s="2" t="n">
-        <v>67.51333333333334</v>
-      </c>
-      <c r="T20" t="n">
-        <v>126.5875</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>HAVELLS</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Havells India Ltd</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>17.06727541291795</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>19.90967741935484</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>6.837009144701453</v>
-      </c>
-      <c r="F21" t="n">
-        <v>10.11834319526627</v>
-      </c>
-      <c r="G21" t="n">
-        <v>8.300161377084454</v>
-      </c>
-      <c r="H21" t="n">
-        <v>10.22279417678758</v>
-      </c>
-      <c r="I21" s="3" t="n">
-        <v>0.040687525177924</v>
-      </c>
-      <c r="J21" s="3" t="n">
-        <v>25.35714285714286</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0.1504518872939926</v>
-      </c>
-      <c r="L21" t="n">
-        <v>335</v>
-      </c>
-      <c r="M21" t="n">
-        <v>17.80967570441255</v>
-      </c>
-      <c r="N21" t="n">
-        <v>1953</v>
-      </c>
-      <c r="O21" s="3" t="n">
-        <v>13.03790793906312</v>
-      </c>
-      <c r="P21" s="4" t="n">
-        <v>10.03323122942004</v>
-      </c>
-      <c r="Q21" s="4" t="n">
-        <v>8.997698704834534</v>
-      </c>
-      <c r="R21" t="n">
-        <v>44</v>
-      </c>
-      <c r="S21" s="2" t="n">
-        <v>1.495214348910158</v>
-      </c>
-      <c r="T21" t="n">
-        <v>4.66148445336008</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>ICICIGI</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>ICICI Lombard General Insurance Company Ltd</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>15.7230643179025</v>
-      </c>
-      <c r="D22" s="2" t="n">
-        <v>145.2287581699346</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>9.366915605017816</v>
-      </c>
-      <c r="F22" t="n">
-        <v>87.42129155073948</v>
-      </c>
-      <c r="G22" t="n">
-        <v>86.76721823595452</v>
-      </c>
-      <c r="H22" t="n">
-        <v>3.031212484993997</v>
-      </c>
-      <c r="I22" s="2" t="n">
-        <v>0.002867677181482999</v>
-      </c>
-      <c r="J22" s="2" t="n">
-        <v>160.0267857142857</v>
-      </c>
-      <c r="K22" t="n">
-        <v>-2.7107202680067</v>
-      </c>
-      <c r="L22" t="n">
-        <v>486</v>
-      </c>
-      <c r="M22" t="n">
-        <v>2.71356783919598</v>
-      </c>
-      <c r="N22" t="n">
-        <v>2407</v>
-      </c>
-      <c r="O22" s="3" t="n">
-        <v>12.91184100336258</v>
-      </c>
-      <c r="P22" s="3" t="n">
-        <v>12.83917371819816</v>
-      </c>
-      <c r="Q22" s="3" t="n">
-        <v>11.1392224868865</v>
-      </c>
-      <c r="R22" t="n">
-        <v>28</v>
-      </c>
-      <c r="S22" s="3" t="n">
-        <v>0.3236083907247109</v>
-      </c>
-      <c r="T22" t="n">
-        <v>22.02903225806451</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>INDIGO</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Interglobe Aviation Ltd</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>892.5683060109289</v>
-      </c>
-      <c r="D23" s="2" t="n">
-        <v>4953.540772532189</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>11.8527226285847</v>
-      </c>
-      <c r="F23" t="n">
-        <v>76.29890862649484</v>
-      </c>
-      <c r="G23" t="n">
-        <v>67.00191570881226</v>
-      </c>
-      <c r="H23" t="n">
-        <v>668.3306055646481</v>
-      </c>
-      <c r="I23" s="2" t="n">
-        <v>0.01857923497267759</v>
-      </c>
-      <c r="J23" s="3" t="n">
-        <v>22.61263972484953</v>
-      </c>
-      <c r="K23" t="n">
-        <v>-0.003252620166245031</v>
-      </c>
-      <c r="L23" t="n">
-        <v>9424</v>
-      </c>
-      <c r="M23" t="n">
-        <v>17.92555113841706</v>
-      </c>
-      <c r="N23" t="n">
-        <v>21183</v>
-      </c>
-      <c r="O23" s="2" t="n">
-        <v>19.31335512580617</v>
-      </c>
-      <c r="P23" s="2" t="n">
-        <v>120.6925086746793</v>
-      </c>
-      <c r="Q23" s="2" t="n">
-        <v>121.2356822276117</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" s="2" t="n">
-        <v>56.38625204582652</v>
-      </c>
-      <c r="T23" t="n">
-        <v>125.7372262773723</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>IRCTC</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Indian Railway Catering &amp; Tourism Corporation Ltd</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>34.39628482972136</v>
-      </c>
-      <c r="D24" s="2" t="n">
-        <v>42.82674772036474</v>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>26.01873536299766</v>
-      </c>
-      <c r="F24" t="n">
-        <v>34.33255269320843</v>
-      </c>
-      <c r="G24" t="n">
-        <v>32.99765807962529</v>
-      </c>
-      <c r="H24" t="n">
-        <v>18.24002626826465</v>
-      </c>
-      <c r="I24" s="2" t="n">
-        <v>0.01857585139318885</v>
-      </c>
-      <c r="J24" s="2" t="n">
-        <v>82.73684210526316</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0.04092769440654843</v>
-      </c>
-      <c r="L24" t="n">
-        <v>667</v>
-      </c>
-      <c r="M24" t="n">
-        <v>45.49795361527968</v>
-      </c>
-      <c r="N24" t="n">
-        <v>882</v>
-      </c>
-      <c r="O24" s="3" t="n">
-        <v>17.95524410389091</v>
-      </c>
-      <c r="P24" s="2" t="n">
-        <v>29.16686408659448</v>
-      </c>
-      <c r="Q24" s="2" t="n">
-        <v>28.47351571234393</v>
-      </c>
-      <c r="R24" t="n">
-        <v>47</v>
-      </c>
-      <c r="S24" s="3" t="n">
-        <v>0.7010343129207027</v>
-      </c>
-      <c r="T24" t="n">
-        <v>12.44897959183673</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>IRFC</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Indian Railway Finance Corporation Ltd</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>13.0380853616381</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>5.746523336036321</v>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>24.0645524488647</v>
-      </c>
-      <c r="F25" t="n">
-        <v>99.50459748545694</v>
-      </c>
-      <c r="G25" t="n">
-        <v>99.47082004128355</v>
-      </c>
-      <c r="H25" t="n">
-        <v>1.321838369595244</v>
-      </c>
-      <c r="I25" s="4" t="n">
-        <v>8.378352548852153</v>
-      </c>
-      <c r="J25" s="4" t="n">
-        <v>1.31948659270683</v>
-      </c>
-      <c r="K25" t="n">
-        <v>15.53898087730547</v>
-      </c>
-      <c r="L25" t="n">
-        <v>7906</v>
-      </c>
-      <c r="M25" t="n">
-        <v>29.81933391166598</v>
-      </c>
-      <c r="N25" t="n">
-        <v>7914</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>19.06740855567788</v>
-      </c>
-      <c r="P25" s="3" t="n">
-        <v>23.24502393394037</v>
-      </c>
-      <c r="Q25" s="3" t="n">
-        <v>20.11244339814313</v>
-      </c>
-      <c r="R25" t="n">
-        <v>31</v>
-      </c>
-      <c r="S25" s="4" t="n">
-        <v>0.05492885738906</v>
-      </c>
-      <c r="T25" t="n">
-        <v>1211.136363636364</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>JIOFIN</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Jio Financial Services Ltd</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="n">
-        <v>1.153456416595399</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>1.104587235082323</v>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>86.52291105121293</v>
-      </c>
-      <c r="F26" t="n">
-        <v>84.04312668463612</v>
-      </c>
-      <c r="G26" t="n">
-        <v>82.85714285714286</v>
-      </c>
-      <c r="H26" t="n">
-        <v>1.107943367181406</v>
-      </c>
-      <c r="I26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="2" t="n">
-        <v>198.8</v>
-      </c>
-      <c r="K26" t="n">
-        <v>-85.49839640795382</v>
-      </c>
-      <c r="L26" t="n">
-        <v>763</v>
-      </c>
-      <c r="M26" t="n">
-        <v>48.94162924951892</v>
-      </c>
-      <c r="N26" t="n">
-        <v>-678</v>
-      </c>
-      <c r="O26" s="4" t="n">
-        <v/>
-      </c>
-      <c r="P26" s="4" t="n">
-        <v/>
-      </c>
-      <c r="Q26" s="4" t="n">
-        <v/>
-      </c>
-      <c r="R26" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" s="4" t="n">
-        <v>0.0128052021565203</v>
-      </c>
-      <c r="T26" t="n">
-        <v>10.78488372093023</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>LODHA</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Macrotech Developers Ltd</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="n">
-        <v>8.895758200240426</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>9.778678428100291</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>15.06397828615743</v>
-      </c>
-      <c r="F27" t="n">
-        <v>25.8336564559907</v>
-      </c>
-      <c r="G27" t="n">
-        <v>23.856145792943</v>
-      </c>
-      <c r="H27" t="n">
-        <v>3.292512394592991</v>
-      </c>
-      <c r="I27" s="3" t="n">
-        <v>0.4406663232010991</v>
-      </c>
-      <c r="J27" s="3" t="n">
-        <v>5.628630705394191</v>
-      </c>
-      <c r="K27" t="n">
-        <v>1.95046904315197</v>
-      </c>
-      <c r="L27" t="n">
-        <v>-435</v>
-      </c>
-      <c r="M27" t="n">
-        <v>-16.32270168855535</v>
-      </c>
-      <c r="N27" t="n">
-        <v>2512</v>
-      </c>
-      <c r="O27" s="4" t="n">
-        <v>-2.827853564186245</v>
-      </c>
-      <c r="P27" s="4" t="n">
-        <v>-1.119685230740497</v>
-      </c>
-      <c r="Q27" s="4" t="n">
-        <v>-5.293423548032761</v>
-      </c>
-      <c r="R27" t="n">
-        <v/>
-      </c>
-      <c r="S27" s="3" t="n">
-        <v>0.2185685834145515</v>
-      </c>
-      <c r="T27" t="n">
-        <v>8.824636441402909</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Larsen &amp; Toubro Ltd</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>77.66510140873214</v>
-      </c>
-      <c r="D28" s="2" t="n">
-        <v>118.5341120014487</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>7.031246466738726</v>
-      </c>
-      <c r="F28" t="n">
-        <v>13.50666853599743</v>
-      </c>
-      <c r="G28" t="n">
-        <v>11.8414566307725</v>
-      </c>
-      <c r="H28" t="n">
-        <v>56.44423467905896</v>
-      </c>
-      <c r="I28" s="3" t="n">
-        <v>0.1034568888000799</v>
-      </c>
-      <c r="J28" s="3" t="n">
-        <v>3.544154751892346</v>
-      </c>
-      <c r="K28" t="n">
-        <v>-0.2234388079691947</v>
-      </c>
-      <c r="L28" t="n">
-        <v>20445</v>
-      </c>
-      <c r="M28" t="n">
-        <v>68.45806127574083</v>
-      </c>
-      <c r="N28" t="n">
-        <v>18266</v>
-      </c>
-      <c r="O28" s="3" t="n">
-        <v>10.33534798968241</v>
-      </c>
-      <c r="P28" s="4" t="n">
-        <v>8.75885858017449</v>
-      </c>
-      <c r="Q28" s="4" t="n">
-        <v>8.561693929531589</v>
-      </c>
-      <c r="R28" t="n">
-        <v>36</v>
-      </c>
-      <c r="S28" s="2" t="n">
-        <v>8.027628521638107</v>
-      </c>
-      <c r="T28" t="n">
-        <v>44.39128689018269</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>MOTHERSON</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Samvardhana Motherson International Ltd</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="n">
-        <v>11.54654941693749</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>11.96258436964212</v>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>3.060025128683176</v>
-      </c>
-      <c r="F29" t="n">
-        <v>9.445547764763102</v>
-      </c>
-      <c r="G29" t="n">
-        <v>5.585052486523731</v>
-      </c>
-      <c r="H29" t="n">
-        <v>3.58763572429851</v>
-      </c>
-      <c r="I29" s="3" t="n">
-        <v>0.7616899254444657</v>
-      </c>
-      <c r="J29" s="3" t="n">
-        <v>5.224737713970182</v>
-      </c>
-      <c r="K29" t="n">
-        <v>1.437567045698348</v>
-      </c>
-      <c r="L29" t="n">
-        <v>925</v>
-      </c>
-      <c r="M29" t="n">
-        <v>9.922763355503111</v>
-      </c>
-      <c r="N29" t="n">
-        <v>7569</v>
-      </c>
-      <c r="O29" s="4" t="n">
-        <v>9.211957132942761</v>
-      </c>
-      <c r="P29" s="4" t="n">
-        <v>7.557399109099472</v>
-      </c>
-      <c r="Q29" s="4" t="n">
-        <v>5.922384104881218</v>
-      </c>
-      <c r="R29" t="n">
-        <v>20</v>
-      </c>
-      <c r="S29" s="3" t="n">
-        <v>1.172420347359167</v>
-      </c>
-      <c r="T29" t="n">
-        <v>3.276409268972844</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>NAUKRI</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Info Edge (India) Ltd</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="n">
-        <v>1.96616218359659</v>
-      </c>
-      <c r="D30" s="4" t="n">
-        <v>1.999475547397404</v>
-      </c>
-      <c r="E30" s="3" t="n">
-        <v>23.46214511041009</v>
-      </c>
-      <c r="F30" t="n">
-        <v>28.03627760252366</v>
-      </c>
-      <c r="G30" t="n">
-        <v>24.05362776025236</v>
-      </c>
-      <c r="H30" t="n">
-        <v>1.648701820499321</v>
-      </c>
-      <c r="I30" s="2" t="n">
-        <v>0.008129006675038002</v>
-      </c>
-      <c r="J30" s="3" t="n">
-        <v>28.97142857142857</v>
-      </c>
-      <c r="K30" t="n">
-        <v>-43.54008438818565</v>
-      </c>
-      <c r="L30" t="n">
-        <v>-150</v>
-      </c>
-      <c r="M30" t="n">
-        <v>-21.09704641350211</v>
-      </c>
-      <c r="N30" t="n">
-        <v>702</v>
-      </c>
-      <c r="O30" s="3" t="n">
-        <v>17.11561008996074</v>
-      </c>
-      <c r="P30" s="4" t="n">
-        <v>0.1011465318701221</v>
-      </c>
-      <c r="Q30" s="4" t="n">
-        <v>-2.129609917599939</v>
-      </c>
-      <c r="R30" t="n">
-        <v>49</v>
-      </c>
-      <c r="S30" s="4" t="n">
-        <v>0.07027071960985341</v>
-      </c>
-      <c r="T30" t="n">
-        <v>3.130864197530864</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>PFC</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Power Finance Corporation Ltd</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>26.1609340860332</v>
-      </c>
-      <c r="D31" s="4" t="n">
-        <v>3.480398875307857</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>28.91659745596014</v>
-      </c>
-      <c r="F31" t="n">
-        <v>36.68859553263103</v>
-      </c>
-      <c r="G31" t="n">
-        <v>36.63067709927001</v>
-      </c>
-      <c r="H31" t="n">
-        <v>2.54707727671322</v>
-      </c>
-      <c r="I31" s="4" t="n">
-        <v>8.521864217426122</v>
-      </c>
-      <c r="J31" s="4" t="n">
-        <v>0.5804147544943239</v>
-      </c>
-      <c r="K31" t="n">
-        <v>25.3474518214041</v>
-      </c>
-      <c r="L31" t="n">
-        <v>-101229</v>
-      </c>
-      <c r="M31" t="n">
-        <v>-301.5190778303994</v>
-      </c>
-      <c r="N31" t="n">
-        <v>-97820</v>
-      </c>
-      <c r="O31" s="3" t="n">
-        <v>11.08175357755092</v>
-      </c>
-      <c r="P31" s="3" t="n">
-        <v>15.92359362270073</v>
-      </c>
-      <c r="Q31" s="3" t="n">
-        <v>14.86983549970351</v>
-      </c>
-      <c r="R31" t="n">
-        <v>23</v>
-      </c>
-      <c r="S31" s="4" t="n">
-        <v>0.0880835748601615</v>
-      </c>
-      <c r="T31" t="n">
-        <v>119.7748691099476</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>PIDILITIND</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Pidilite Industries Ltd</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>20.78030212917806</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>26.93139151211742</v>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>14.10805136073649</v>
-      </c>
-      <c r="F32" t="n">
-        <v>21.86869094726642</v>
-      </c>
-      <c r="G32" t="n">
-        <v>19.11491561011064</v>
-      </c>
-      <c r="H32" t="n">
-        <v>14.46671083140112</v>
-      </c>
-      <c r="I32" s="3" t="n">
-        <v>0.04543832520518615</v>
-      </c>
-      <c r="J32" s="3" t="n">
-        <v>54.33333333333334</v>
-      </c>
-      <c r="K32" t="n">
-        <v>-0.6842688330871491</v>
-      </c>
-      <c r="L32" t="n">
-        <v>955</v>
-      </c>
-      <c r="M32" t="n">
-        <v>35.2658788774003</v>
-      </c>
-      <c r="N32" t="n">
-        <v>2724</v>
-      </c>
-      <c r="O32" s="3" t="n">
-        <v>11.83637017589811</v>
-      </c>
-      <c r="P32" s="3" t="n">
-        <v>13.48774998597666</v>
-      </c>
-      <c r="Q32" s="3" t="n">
-        <v>13.56415724960776</v>
-      </c>
-      <c r="R32" t="n">
-        <v>47</v>
-      </c>
-      <c r="S32" s="3" t="n">
-        <v>1.025422325273269</v>
-      </c>
-      <c r="T32" t="n">
-        <v>2.271693267290405</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>RECLTD</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>REC Ltd</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>20.39653929343908</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>9.294489608054098</v>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>29.7682934528695</v>
-      </c>
-      <c r="F33" t="n">
-        <v>100.7702506471368</v>
-      </c>
-      <c r="G33" t="n">
-        <v>100.7197424079803</v>
-      </c>
-      <c r="H33" t="n">
-        <v>2.580305039666831</v>
-      </c>
-      <c r="I33" s="4" t="n">
-        <v>6.424917087238645</v>
-      </c>
-      <c r="J33" s="4" t="n">
-        <v>1.600474155202351</v>
-      </c>
-      <c r="K33" t="n">
-        <v>9.193576008186621</v>
-      </c>
-      <c r="L33" t="n">
-        <v>-59554</v>
-      </c>
-      <c r="M33" t="n">
-        <v>-124.3739949460142</v>
-      </c>
-      <c r="N33" t="n">
-        <v>-57723</v>
-      </c>
-      <c r="O33" s="3" t="n">
-        <v>13.33804224786568</v>
-      </c>
-      <c r="P33" s="3" t="n">
-        <v>19.76311435023079</v>
-      </c>
-      <c r="Q33" s="3" t="n">
-        <v>19.67245924901726</v>
-      </c>
-      <c r="R33" t="n">
-        <v>30</v>
-      </c>
-      <c r="S33" s="4" t="n">
-        <v>0.08667964267928514</v>
-      </c>
-      <c r="T33" t="n">
-        <v>75.18512658227849</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>SHREECEM</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Shree Cement Ltd</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="n">
-        <v>8.370767521615225</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>11.72234894226039</v>
-      </c>
-      <c r="E34" s="3" t="n">
-        <v>8.445007553238145</v>
-      </c>
-      <c r="F34" t="n">
-        <v>22.01647093221578</v>
-      </c>
-      <c r="G34" t="n">
-        <v>12.77228205253155</v>
-      </c>
-      <c r="H34" t="n">
-        <v>6.205908683974934</v>
-      </c>
-      <c r="I34" s="3" t="n">
-        <v>0.07998840747717723</v>
-      </c>
-      <c r="J34" s="3" t="n">
-        <v>19.82558139534884</v>
-      </c>
-      <c r="K34" t="n">
-        <v>-1.305887560867641</v>
-      </c>
-      <c r="L34" t="n">
-        <v>1929</v>
-      </c>
-      <c r="M34" t="n">
-        <v>42.69588313413015</v>
-      </c>
-      <c r="N34" t="n">
-        <v>3347</v>
-      </c>
-      <c r="O34" s="3" t="n">
-        <v>10.32561591555659</v>
-      </c>
-      <c r="P34" s="4" t="n">
-        <v>11.2926552609119</v>
-      </c>
-      <c r="Q34" s="4" t="n">
-        <v>10.67987982673917</v>
-      </c>
-      <c r="R34" t="n">
-        <v>16</v>
-      </c>
-      <c r="S34" s="3" t="n">
-        <v>0.7348612354521038</v>
-      </c>
-      <c r="T34" t="n">
-        <v>2.139610051089563</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>TITAN</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Titan Company Ltd
-</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>37.2192057915469</v>
-      </c>
-      <c r="D35" s="3" t="n">
-        <v>18.8916977649372</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>6.843630099444054</v>
-      </c>
-      <c r="F35" t="n">
-        <v>10.35940803382664</v>
-      </c>
-      <c r="G35" t="n">
-        <v>9.21619293712317</v>
-      </c>
-      <c r="H35" t="n">
-        <v>11.08187783307446</v>
-      </c>
-      <c r="I35" s="4" t="n">
-        <v>1.653145959757266</v>
-      </c>
-      <c r="J35" s="3" t="n">
-        <v>9.411954765751211</v>
-      </c>
-      <c r="K35" t="n">
-        <v>2.491118669690098</v>
-      </c>
-      <c r="L35" t="n">
-        <v>1506</v>
-      </c>
-      <c r="M35" t="n">
-        <v>28.45804988662132</v>
-      </c>
-      <c r="N35" t="n">
-        <v>1695</v>
-      </c>
-      <c r="O35" s="2" t="n">
-        <v>20.89716395312024</v>
-      </c>
-      <c r="P35" s="3" t="n">
-        <v>20.27457629679304</v>
-      </c>
-      <c r="Q35" s="3" t="n">
-        <v>19.50578386760935</v>
-      </c>
-      <c r="R35" t="n">
-        <v>28</v>
-      </c>
-      <c r="S35" s="2" t="n">
-        <v>1.619298190002219</v>
-      </c>
-      <c r="T35" t="n">
-        <v>13.77298463197627</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>TRENT</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Trent Ltd</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>36.30776794493609</v>
-      </c>
-      <c r="D36" s="3" t="n">
-        <v>22.33293248582718</v>
-      </c>
-      <c r="E36" s="3" t="n">
-        <v>11.93535353535353</v>
-      </c>
-      <c r="F36" t="n">
-        <v>15.92727272727273</v>
-      </c>
-      <c r="G36" t="n">
-        <v>10.50505050505051</v>
-      </c>
-      <c r="H36" t="n">
-        <v>20.62273108070371</v>
-      </c>
-      <c r="I36" s="3" t="n">
-        <v>0.4309242871189774</v>
-      </c>
-      <c r="J36" s="3" t="n">
-        <v>8.043478260869565</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0.1709791983764586</v>
-      </c>
-      <c r="L36" t="n">
-        <v>841</v>
-      </c>
-      <c r="M36" t="n">
-        <v>42.66869609335362</v>
-      </c>
-      <c r="N36" t="n">
-        <v>1349</v>
-      </c>
-      <c r="O36" s="2" t="n">
-        <v>36.30691600183056</v>
-      </c>
-      <c r="P36" s="2" t="n">
-        <v>73.11367578503176</v>
-      </c>
-      <c r="Q36" s="2" t="n">
-        <v>69.52182030724354</v>
-      </c>
-      <c r="R36" t="n">
-        <v>8</v>
-      </c>
-      <c r="S36" s="2" t="n">
-        <v>1.727869310248534</v>
-      </c>
-      <c r="T36" t="n">
-        <v>5.051020408163265</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr"/>
-      <c r="B37" s="1" t="inlineStr">
-        <is>
-          <t>Peer Group Median</t>
-        </is>
-      </c>
-      <c r="C37" s="1" t="n">
-        <v>15.7230643179025</v>
-      </c>
-      <c r="D37" s="1" t="n">
-        <v>12.99549647732646</v>
-      </c>
-      <c r="E37" s="1" t="n">
-        <v>14.28829915560917</v>
-      </c>
-      <c r="F37" s="1" t="n">
-        <v>24.92105782514308</v>
-      </c>
-      <c r="G37" s="1" t="n">
-        <v>23.62797059326381</v>
-      </c>
-      <c r="H37" s="1" t="n">
-        <v>6.926554927819896</v>
-      </c>
-      <c r="I37" s="1" t="n">
-        <v>0.3623864473361159</v>
-      </c>
-      <c r="J37" s="1" t="n">
-        <v>10.5045045045045</v>
-      </c>
-      <c r="K37" s="1" t="n">
-        <v>0.1181198246468583</v>
-      </c>
-      <c r="L37" s="1" t="n">
-        <v>883</v>
-      </c>
-      <c r="M37" s="1" t="n">
-        <v>18.26629387877874</v>
-      </c>
-      <c r="N37" s="1" t="n">
-        <v>2631.5</v>
-      </c>
-      <c r="O37" s="1" t="n">
-        <v>13.0337841442581</v>
-      </c>
-      <c r="P37" s="1" t="n">
-        <v>19.39426501332384</v>
-      </c>
-      <c r="Q37" s="1" t="n">
-        <v>17.91008294870988</v>
-      </c>
-      <c r="R37" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="S37" s="1" t="n">
-        <v>0.6018691588785047</v>
-      </c>
-      <c r="T37" s="1" t="n">
-        <v>5.051020408163265</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>